<commit_message>
updated data (more cases)
</commit_message>
<xml_diff>
--- a/data/pv_data_sample.xlsx
+++ b/data/pv_data_sample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rohit\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08EF1350-F43D-426D-9575-E7BDA8C2E9DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DCBDF99-21C5-4CA4-9C8E-0F625FD3070A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="273">
   <si>
     <t>Condition_ID</t>
   </si>
@@ -484,7 +484,361 @@
     <t>80% mismatch row1-8 col1, R=15</t>
   </si>
   <si>
-    <t>Condition:(1PS)/(2MM)/(3Normal)</t>
+    <t>Condition:(1PS)/(2MM)/(3Normal)/(4CrossString)</t>
+  </si>
+  <si>
+    <t>3.558e + 02</t>
+  </si>
+  <si>
+    <t>6.054e + 03</t>
+  </si>
+  <si>
+    <t>2.766e + 02</t>
+  </si>
+  <si>
+    <t>2.189e + 01</t>
+  </si>
+  <si>
+    <t>3.626e + 02</t>
+  </si>
+  <si>
+    <t>6.369e + 03</t>
+  </si>
+  <si>
+    <t>2.888e + 02</t>
+  </si>
+  <si>
+    <t>2.205e + 01</t>
+  </si>
+  <si>
+    <t>3.631e + 02</t>
+  </si>
+  <si>
+    <t>2.907e + 02</t>
+  </si>
+  <si>
+    <t>2.191e + 01</t>
+  </si>
+  <si>
+    <t>2.878e + 02</t>
+  </si>
+  <si>
+    <t>2.213e + 01</t>
+  </si>
+  <si>
+    <t>2.883e + 02</t>
+  </si>
+  <si>
+    <t>2.209e + 01</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-6 )-2(col2 , row1-5) R=0.000001</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-3 )-2(col2 , row1-8) R=0.000001</t>
+  </si>
+  <si>
+    <t>2.212e + 02</t>
+  </si>
+  <si>
+    <t>3.412e + 03</t>
+  </si>
+  <si>
+    <t>1.566e + 02</t>
+  </si>
+  <si>
+    <t>2.178e + 01</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-3 )-2(col2 , row1-8) R=1</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-3 )-2(col2 , row1-8) R=5</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-3 )-2(col2 , row1-8) R=15</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-3 )-2(col2 , row1-8) R=10</t>
+  </si>
+  <si>
+    <t>3.448e + 03</t>
+  </si>
+  <si>
+    <t>2.161e + 01</t>
+  </si>
+  <si>
+    <t>2.431e + 02</t>
+  </si>
+  <si>
+    <t>3.184e + 02</t>
+  </si>
+  <si>
+    <t>3.654e + 03</t>
+  </si>
+  <si>
+    <t>1.795e + 02</t>
+  </si>
+  <si>
+    <t>2.036e + 01</t>
+  </si>
+  <si>
+    <t>3.437e + 02</t>
+  </si>
+  <si>
+    <t>4.082e + 03</t>
+  </si>
+  <si>
+    <t>2.285e + 02</t>
+  </si>
+  <si>
+    <t>1.786e + 01</t>
+  </si>
+  <si>
+    <t>3.500e + 02</t>
+  </si>
+  <si>
+    <t>4.563e + 03</t>
+  </si>
+  <si>
+    <t>2.669e + 02</t>
+  </si>
+  <si>
+    <t>1.710e + 01</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-1 )-2(col3 , row1-1) R=15</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-1 )-2(col3 , row1-1) R=10</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-1 )-2(col3 , row1-1) R=5</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-1 )-2(col3 , row1-1) R=1</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-1 )-2(col3 , row1-1) R=0.000001</t>
+  </si>
+  <si>
+    <t>2.897e + 02</t>
+  </si>
+  <si>
+    <t>2.198e + 01</t>
+  </si>
+  <si>
+    <t>2.902e + 02</t>
+  </si>
+  <si>
+    <t>2.194e + 01</t>
+  </si>
+  <si>
+    <t>6.361e + 03</t>
+  </si>
+  <si>
+    <t>2.854e + 02</t>
+  </si>
+  <si>
+    <t>2.229e + 01</t>
+  </si>
+  <si>
+    <t>Cross String  1(col1 , row1-5 )-2(col2 , row1-5) R=1</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-5 )-2(col2 , row1-5) R=5</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-5 )-2(col2 , row1-5) R=10</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-5 )-2(col2 , row1-5) R=15</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-9 )-2(col3 , row1-9) R=0.000001</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-9 )-2(col3 , row1-9) R=1</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-9 )-2(col3 , row1-9) R=5</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-9 )-2(col3 , row1-9) R=10</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row1-9 )-2(col3 , row1-9) R=15</t>
+  </si>
+  <si>
+    <t>6.457e + 03</t>
+  </si>
+  <si>
+    <t>2.927e + 02</t>
+  </si>
+  <si>
+    <t>2.206e + 01</t>
+  </si>
+  <si>
+    <t>3.743e + 02</t>
+  </si>
+  <si>
+    <t>3.757e + 02</t>
+  </si>
+  <si>
+    <t>6.444e + 03</t>
+  </si>
+  <si>
+    <t>2.235e + 01</t>
+  </si>
+  <si>
+    <t>6.468e + 03</t>
+  </si>
+  <si>
+    <t>2.946e + 02</t>
+  </si>
+  <si>
+    <t>2.195e + 01</t>
+  </si>
+  <si>
+    <t>3.791e + 02</t>
+  </si>
+  <si>
+    <t>3.801e + 02</t>
+  </si>
+  <si>
+    <t>6.463e + 03</t>
+  </si>
+  <si>
+    <t>2.985e + 02</t>
+  </si>
+  <si>
+    <t>2.165e + 01</t>
+  </si>
+  <si>
+    <t>6.481e + 03</t>
+  </si>
+  <si>
+    <t>2.941e + 02</t>
+  </si>
+  <si>
+    <t>3.811e + 02</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row0-0 )-2(col3 , row0-0) R=0.000001</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row0-0 )-2(col3 , row0-0) R=1</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row0-0 )-2(col3 , row0-0) R=5</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row0-0 )-2(col3 , row0-0) R=10</t>
+  </si>
+  <si>
+    <t>Cross String 1(col1 , row0-0 )-2(col3 , row0-0) R=15</t>
+  </si>
+  <si>
+    <t>6.520e + 03</t>
+  </si>
+  <si>
+    <t>2.217e + 01</t>
+  </si>
+  <si>
+    <t>3.825e + 02</t>
+  </si>
+  <si>
+    <t>3.830e + 02</t>
+  </si>
+  <si>
+    <t>6.521e + 03</t>
+  </si>
+  <si>
+    <t>2.936e + 02</t>
+  </si>
+  <si>
+    <t>2.221e + 01</t>
+  </si>
+  <si>
+    <t>PS rows1–10 col1, 8000W/m2</t>
+  </si>
+  <si>
+    <t>PS rows1–10 col1, 600W/m2</t>
+  </si>
+  <si>
+    <t>PS rows1–10 col1, 400W/m2</t>
+  </si>
+  <si>
+    <t>PS rows1–10 col1, 200W/m2</t>
+  </si>
+  <si>
+    <t>PS rows1–10 col1, 0W/m2</t>
+  </si>
+  <si>
+    <t>6.124e + 03</t>
+  </si>
+  <si>
+    <t>2.975e + 02</t>
+  </si>
+  <si>
+    <t>2.058e + 01</t>
+  </si>
+  <si>
+    <t>2.820e + 02</t>
+  </si>
+  <si>
+    <t>5.703e + 03</t>
+  </si>
+  <si>
+    <t>2.961e + 02</t>
+  </si>
+  <si>
+    <t>3.806e + 02</t>
+  </si>
+  <si>
+    <t>3.796e + 02</t>
+  </si>
+  <si>
+    <t>5.276e + 03</t>
+  </si>
+  <si>
+    <t>2.999e + 02</t>
+  </si>
+  <si>
+    <t>1.759e + 01</t>
+  </si>
+  <si>
+    <t>4.836e + 03</t>
+  </si>
+  <si>
+    <t>2.995e + 02</t>
+  </si>
+  <si>
+    <t>1.615e + 01</t>
+  </si>
+  <si>
+    <t>1.730e + 01</t>
+  </si>
+  <si>
+    <t>3.781e + 02</t>
+  </si>
+  <si>
+    <t>1.887e + 01</t>
+  </si>
+  <si>
+    <t>2.045e + 01</t>
+  </si>
+  <si>
+    <t>2.202e + 01</t>
+  </si>
+  <si>
+    <t>1.573e + 01</t>
+  </si>
+  <si>
+    <t>4.389e + 03</t>
+  </si>
+  <si>
+    <t>1.470e + 01</t>
   </si>
 </sst>
 </file>
@@ -881,12 +1235,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" customWidth="1"/>
     <col min="2" max="2" width="24.85546875" customWidth="1"/>
-    <col min="3" max="3" width="40.42578125" customWidth="1"/>
+    <col min="3" max="3" width="56.28515625" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="13.7109375" customWidth="1"/>
     <col min="6" max="6" width="14.140625" customWidth="1"/>
@@ -1981,6 +2335,1056 @@
         <v>15</v>
       </c>
     </row>
+    <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>4</v>
+      </c>
+      <c r="C32" t="s">
+        <v>170</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I32" s="5">
+        <v>25</v>
+      </c>
+      <c r="J32" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K32" s="5">
+        <v>9.9999999999999995E-7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>4</v>
+      </c>
+      <c r="C33" t="s">
+        <v>207</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I33" s="5">
+        <v>25</v>
+      </c>
+      <c r="J33" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K33" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>4</v>
+      </c>
+      <c r="C34" t="s">
+        <v>208</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I34" s="5">
+        <v>25</v>
+      </c>
+      <c r="J34" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K34" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>4</v>
+      </c>
+      <c r="C35" t="s">
+        <v>209</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I35" s="5">
+        <v>25</v>
+      </c>
+      <c r="J35" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K35" s="5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>4</v>
+      </c>
+      <c r="C36" t="s">
+        <v>210</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I36" s="5">
+        <v>25</v>
+      </c>
+      <c r="J36" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K36" s="5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>4</v>
+      </c>
+      <c r="C37" t="s">
+        <v>171</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I37" s="5">
+        <v>25</v>
+      </c>
+      <c r="J37" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K37" s="5">
+        <v>9.9999999999999995E-7</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>4</v>
+      </c>
+      <c r="C38" t="s">
+        <v>176</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I38" s="5">
+        <v>25</v>
+      </c>
+      <c r="J38" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K38" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>4</v>
+      </c>
+      <c r="C39" t="s">
+        <v>177</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I39" s="5">
+        <v>25</v>
+      </c>
+      <c r="J39" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K39" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>4</v>
+      </c>
+      <c r="C40" t="s">
+        <v>179</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I40" s="5">
+        <v>25</v>
+      </c>
+      <c r="J40" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K40" s="5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>4</v>
+      </c>
+      <c r="C41" t="s">
+        <v>178</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I41" s="5">
+        <v>25</v>
+      </c>
+      <c r="J41" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K41" s="5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>4</v>
+      </c>
+      <c r="C42" t="s">
+        <v>199</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I42" s="5">
+        <v>25</v>
+      </c>
+      <c r="J42" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K42" s="5">
+        <v>9.9999999999999995E-7</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>4</v>
+      </c>
+      <c r="C43" t="s">
+        <v>198</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I43" s="5">
+        <v>25</v>
+      </c>
+      <c r="J43" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K43" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>4</v>
+      </c>
+      <c r="C44" t="s">
+        <v>197</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="G44" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="H44" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I44" s="5">
+        <v>25</v>
+      </c>
+      <c r="J44" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K44" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>4</v>
+      </c>
+      <c r="C45" t="s">
+        <v>196</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I45" s="5">
+        <v>25</v>
+      </c>
+      <c r="J45" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K45" s="5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <v>4</v>
+      </c>
+      <c r="C46" t="s">
+        <v>195</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="H46" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I46" s="5">
+        <v>25</v>
+      </c>
+      <c r="J46" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K46" s="5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <v>4</v>
+      </c>
+      <c r="C47" t="s">
+        <v>211</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I47" s="5">
+        <v>25</v>
+      </c>
+      <c r="J47" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K47" s="5">
+        <v>9.9999999999999995E-7</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48">
+        <v>4</v>
+      </c>
+      <c r="C48" t="s">
+        <v>212</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="G48" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="H48" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I48" s="5">
+        <v>25</v>
+      </c>
+      <c r="J48" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K48" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49">
+        <v>4</v>
+      </c>
+      <c r="C49" t="s">
+        <v>213</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="G49" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="H49" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I49" s="5">
+        <v>25</v>
+      </c>
+      <c r="J49" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K49" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50">
+        <v>4</v>
+      </c>
+      <c r="C50" t="s">
+        <v>214</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="G50" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="H50" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I50" s="5">
+        <v>25</v>
+      </c>
+      <c r="J50" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K50" s="5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51">
+        <v>4</v>
+      </c>
+      <c r="C51" t="s">
+        <v>215</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I51" s="5">
+        <v>25</v>
+      </c>
+      <c r="J51" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K51" s="5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52">
+        <v>4</v>
+      </c>
+      <c r="C52" t="s">
+        <v>234</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="G52" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I52" s="5">
+        <v>25</v>
+      </c>
+      <c r="J52" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K52" s="5">
+        <v>9.9999999999999995E-7</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53">
+        <v>4</v>
+      </c>
+      <c r="C53" t="s">
+        <v>235</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="G53" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="H53" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I53" s="5">
+        <v>25</v>
+      </c>
+      <c r="J53" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K53" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54">
+        <v>4</v>
+      </c>
+      <c r="C54" t="s">
+        <v>236</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="H54" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I54" s="5">
+        <v>25</v>
+      </c>
+      <c r="J54" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K54" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55">
+        <v>4</v>
+      </c>
+      <c r="C55" t="s">
+        <v>237</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="H55" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I55" s="5">
+        <v>25</v>
+      </c>
+      <c r="J55" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K55" s="5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56">
+        <v>4</v>
+      </c>
+      <c r="C56" t="s">
+        <v>238</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="H56" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I56" s="5">
+        <v>25</v>
+      </c>
+      <c r="J56" s="5">
+        <v>1000</v>
+      </c>
+      <c r="K56" s="5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57" t="s">
+        <v>246</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="F57" t="s">
+        <v>253</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="I57">
+        <v>25</v>
+      </c>
+      <c r="J57">
+        <v>1000</v>
+      </c>
+      <c r="K57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58">
+        <v>1</v>
+      </c>
+      <c r="C58" t="s">
+        <v>247</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="E58" t="s">
+        <v>256</v>
+      </c>
+      <c r="F58" t="s">
+        <v>26</v>
+      </c>
+      <c r="G58" t="s">
+        <v>257</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="I58">
+        <v>25</v>
+      </c>
+      <c r="J58">
+        <v>600</v>
+      </c>
+      <c r="K58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>248</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="I59">
+        <v>25</v>
+      </c>
+      <c r="J59">
+        <v>400</v>
+      </c>
+      <c r="K59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>249</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="I60">
+        <v>25</v>
+      </c>
+      <c r="J60">
+        <v>200</v>
+      </c>
+      <c r="K60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>250</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="I61">
+        <v>25</v>
+      </c>
+      <c r="J61">
+        <v>0</v>
+      </c>
+      <c r="K61">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>